<commit_message>
Hoàn tất Flow + Hình ảnh
</commit_message>
<xml_diff>
--- a/server/review_data/xuatnhapcanh/question.xlsx
+++ b/server/review_data/xuatnhapcanh/question.xlsx
@@ -1,43 +1,60 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23801"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\HTML CSS JAVASCRIPT\CCHC\server\review_data\xuatnhapcanh\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5764F9D6-2AD5-4476-94EF-4F87E8FD04DE}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+  <si>
+    <t>question</t>
+  </si>
+  <si>
+    <t>answer</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,94 +62,29 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -420,65 +372,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>question</t>
-        </is>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Hỗ trợ tôi cấp Căn cước</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Cám ơn bạn! Tôi có thể hỗ trợ bạn cấp Căn cước cho số lượng người và địa điểm bạn yêu cầu. 
-Bạn có thể cung cấp thông tin về:
-* Số lượng người cần cấp Căn cước
-* địa điểm cần cấp Căn cước
-* loại Căn cước bạn muốn mua (ví dụ: Giấy, thẻ,...)
-Tôi sẽ giúp bạn chọn Căn cước phù hợp và cấp cho bạn trong thời gian sớm nhất có thể.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Hỗ trợ tôi cấp Căn cước</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Cảm ơn bạn. Vui lòng cho tôi biết cụ thể việc cần cấp căn cước và tôi sẽ hỗ trợ bạn trong tối thiểu 24 giờ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Hô trợ tôi quy trình cấp họ chiếu</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Cám ơn bạn đã đặt câu hỏi. Để giúp bạn quy trình cấp họ chiếu, vui lòng cung cấp cho tôi thông tin về họ, chi tiết liên quan đến việc chiếu và các yêu cầu của họ.</t>
-        </is>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>